<commit_message>
Revisão geral R4 (parte 1): tabela de ataques com coluna "Estado atual" (deteção e mitigação separadas), política de registo e monitorização §4 corrigida (riscos #4 e #7 pós-Fase 9, risco #10, incoerência nível 10 vs revisão semanal)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Lk2S9R4Pvx1JAK73UPgK7J
</commit_message>
<xml_diff>
--- a/tabela-resumo-ataques.xlsx
+++ b/tabela-resumo-ataques.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ataques do Lab" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Ataques do Lab'!$A$1:$N$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Ataques do Lab'!$A$2:$O$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,6 +41,10 @@
     <font>
       <name val="Arial"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <i val="1"/>
     </font>
   </fonts>
   <fills count="7">
@@ -107,7 +111,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -133,6 +137,7 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -498,7 +503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N20"/>
+  <dimension ref="A1:O21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -515,171 +520,112 @@
     <col width="34" customWidth="1" min="12" max="12"/>
     <col width="42" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="60" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Ataque / Ameaça</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Tipo</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Descrição breve</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Objetivo</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Gravidade</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Impacto</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Indicadores / Sinais</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Prevenção</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Deteção</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Resposta / Mitigação</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Mecanismos / Ferramentas de defesa</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>ISO 27001 / NIS2 / RGPD</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Exemplo</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Prioridade de estudo</t>
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>Nota (revisão de 2026-10-20): As colunas originais descrevem o estado no momento do ataque (até à Fase 6). O estado atual da deteção está no mapa-cobertura-mitre-attack.md; a coluna 'Estado atual' resume-o, com a evidência mais recente.</t>
         </is>
       </c>
     </row>
     <row r="2" ht="110" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>SQL Injection</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>Ataque a aplicações web (injeção de código)</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>Inserção de comandos SQL não intencionados através de campos de input não validados, alterando a lógica da query original.</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>Aceder, extrair, alterar ou apagar dados da base de dados; contornar autenticação.</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>Crítica</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>Confidencialidade, Integridade</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>Erros de sintaxe SQL devolvidos ao utilizador; padrões `' OR '1'='1`, comentários SQL (--, #) em parâmetros; tempos de resposta anómalos (blind/time-based).</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>Prepared statements / queries parametrizadas (defesa definitiva, não um "modo"); validação de tipo de input; princípio do menor privilégio na conta de BD.</t>
-        </is>
-      </c>
-      <c r="I2" s="3" t="inlineStr">
-        <is>
-          <t>WAF com assinaturas de SQLi; monitorização de queries anómalas; logs de erro da base de dados.</t>
-        </is>
-      </c>
-      <c r="J2" s="3" t="inlineStr">
-        <is>
-          <t>Isolar o servidor, rever/rodar credenciais da BD, procurar sinais de exfiltração, avaliar notificação de violação se houver dados pessoais expostos.</t>
-        </is>
-      </c>
-      <c r="K2" s="3" t="inlineStr">
-        <is>
-          <t>WAF, prepared statements, ORM seguro, princípio do menor privilégio na conta de BD.</t>
-        </is>
-      </c>
-      <c r="L2" s="3" t="inlineStr">
-        <is>
-          <t>ISO 27001 A.8.28 (codificação segura), A.8.25 (ciclo de desenvolvimento seguro); NIS2 Art.21; RGPD (notificação de violação se dados pessoais expostos).</t>
-        </is>
-      </c>
-      <c r="M2" s="3" t="inlineStr">
-        <is>
-          <t>Entrada #16 — payload 1' OR '1'='1' # devolveu os 5 utilizadores no nível High; bloqueado no Impossible por prepared statements.</t>
-        </is>
-      </c>
-      <c r="N2" s="5" t="inlineStr">
-        <is>
-          <t>⭐⭐⭐</t>
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Ataque / Ameaça</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>Descrição breve</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>Objetivo</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>Gravidade</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>Impacto</t>
+        </is>
+      </c>
+      <c r="G2" s="1" t="inlineStr">
+        <is>
+          <t>Indicadores / Sinais</t>
+        </is>
+      </c>
+      <c r="H2" s="1" t="inlineStr">
+        <is>
+          <t>Prevenção</t>
+        </is>
+      </c>
+      <c r="I2" s="1" t="inlineStr">
+        <is>
+          <t>Deteção</t>
+        </is>
+      </c>
+      <c r="J2" s="1" t="inlineStr">
+        <is>
+          <t>Resposta / Mitigação</t>
+        </is>
+      </c>
+      <c r="K2" s="1" t="inlineStr">
+        <is>
+          <t>Mecanismos / Ferramentas de defesa</t>
+        </is>
+      </c>
+      <c r="L2" s="1" t="inlineStr">
+        <is>
+          <t>ISO 27001 / NIS2 / RGPD</t>
+        </is>
+      </c>
+      <c r="M2" s="1" t="inlineStr">
+        <is>
+          <t>Exemplo</t>
+        </is>
+      </c>
+      <c r="N2" s="1" t="inlineStr">
+        <is>
+          <t>Prioridade de estudo</t>
+        </is>
+      </c>
+      <c r="O2" s="1" t="inlineStr">
+        <is>
+          <t>Estado atual no lab (2026-10-20)</t>
         </is>
       </c>
     </row>
     <row r="3" ht="110" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Command Injection</t>
+          <t>SQL Injection</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Ataque a aplicações web (injeção de comandos SO)</t>
+          <t>Ataque a aplicações web (injeção de código)</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Injeção de comandos do sistema operativo através de um input processado por uma função que invoca a shell.</t>
+          <t>Inserção de comandos SQL não intencionados através de campos de input não validados, alterando a lógica da query original.</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Execução de comandos arbitrários no servidor (RCE); controlo do sistema operativo subjacente.</t>
+          <t>Aceder, extrair, alterar ou apagar dados da base de dados; contornar autenticação.</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
@@ -689,104 +635,109 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Confidencialidade, Integridade, Disponibilidade</t>
+          <t>Confidencialidade, Integridade</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Caracteres de encadeamento de shell (; &amp; | &amp;&amp;) em parâmetros de input; processos filho inesperados do processo web; picos de CPU inexplicados (cryptomining).</t>
+          <t>Erros de sintaxe SQL devolvidos ao utilizador; padrões `' OR '1'='1`, comentários SQL (--, #) em parâmetros; tempos de resposta anómalos (blind/time-based).</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Whitelist estrita de formato de input (nunca blacklist de caracteres); evitar chamadas diretas à shell; sandboxing/containers com privilégios mínimos.</t>
+          <t>Prepared statements / queries parametrizadas (defesa definitiva, não um "modo"); validação de tipo de input; princípio do menor privilégio na conta de BD.</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>EDR a monitorizar processos filho anómalos de processos web; IDS/IPS com assinaturas.</t>
+          <t>WAF com assinaturas de SQLi; monitorização de queries anómalas; logs de erro da base de dados.</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>Isolar o servidor, terminar processos maliciosos, procurar persistência/backdoors instalados, reconstruir a partir de imagem limpa se comprometido.</t>
+          <t>Isolar o servidor, rever/rodar credenciais da BD, procurar sinais de exfiltração, avaliar notificação de violação se houver dados pessoais expostos.</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>WAF, EDR, whitelisting de input, princípio do menor privilégio no utilizador de serviço.</t>
+          <t>WAF, prepared statements, ORM seguro, princípio do menor privilégio na conta de BD.</t>
         </is>
       </c>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t>ISO 27001 A.8.28; NIS2 Art.21.</t>
+          <t>ISO 27001 A.8.28 (codificação segura), A.8.25 (ciclo de desenvolvimento seguro); NIS2 Art.21; RGPD (notificação de violação se dados pessoais expostos).</t>
         </is>
       </c>
       <c r="M3" s="3" t="inlineStr">
         <is>
-          <t>Entrada #20 — bypasses do High (&amp;, |) bloqueados no Impossible por whitelist de formato IP; resultado sempre idêntico para qualquer input inválido, assinatura de whitelist.</t>
+          <t>Entrada #16 — payload 1' OR '1'='1' # devolveu os 5 utilizadores no nível High; bloqueado no Impossible por prepared statements.</t>
         </is>
       </c>
       <c r="N3" s="5" t="inlineStr">
         <is>
           <t>⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="O3" s="3" t="inlineStr">
+        <is>
+          <t>Deteção: 🔴 (mapa MITRE); Fase 10: verificar se o Suricata o deteta (gatilho do risco #10). Mitigação: nenhuma no lab — o DVWA é vulnerável de propósito (a defesa correta está na coluna "Prevenção" e no nível Impossible).</t>
         </is>
       </c>
     </row>
     <row r="4" ht="110" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>XSS Reflected</t>
+          <t>Command Injection</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Ataque a aplicações web (injeção de script, client-side)</t>
+          <t>Ataque a aplicações web (injeção de comandos SO)</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Script malicioso refletido de volta na resposta HTTP e executado no browser da vítima; exige que a vítima clique num link preparado.</t>
+          <t>Injeção de comandos do sistema operativo através de um input processado por uma função que invoca a shell.</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Sequestro de sessão, phishing dentro de um domínio de confiança, entrega de malware.</t>
-        </is>
-      </c>
-      <c r="E4" s="6" t="inlineStr">
-        <is>
-          <t>Média-Alta</t>
+          <t>Execução de comandos arbitrários no servidor (RCE); controlo do sistema operativo subjacente.</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Crítica</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Confidencialidade (sessão/cookies), Integridade (ações em nome da vítima)</t>
+          <t>Confidencialidade, Integridade, Disponibilidade</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Parâmetros de URL com tags HTML/JS; violações de CSP registadas; relatos de utilizadores sobre comportamento estranho ao clicar num link.</t>
+          <t>Caracteres de encadeamento de shell (; &amp; | &amp;&amp;) em parâmetros de input; processos filho inesperados do processo web; picos de CPU inexplicados (cryptomining).</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Output encoding de todo o conteúdo gerado a partir de input do utilizador; Content Security Policy (CSP); cookies HttpOnly.</t>
+          <t>Whitelist estrita de formato de input (nunca blacklist de caracteres); evitar chamadas diretas à shell; sandboxing/containers com privilégios mínimos.</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>WAF; CSP com relatório de violações (report-uri); formação de utilizadores.</t>
+          <t>EDR a monitorizar processos filho anómalos de processos web; IDS/IPS com assinaturas.</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>Invalidar sessões ativas, notificar utilizadores afetados, corrigir o encoding em falta.</t>
+          <t>Isolar o servidor, terminar processos maliciosos, procurar persistência/backdoors instalados, reconstruir a partir de imagem limpa se comprometido.</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Output encoding, CSP, HttpOnly, WAF.</t>
+          <t>WAF, EDR, whitelisting de input, princípio do menor privilégio no utilizador de serviço.</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
@@ -796,213 +747,228 @@
       </c>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>Entrada #24 — payload &lt;img src=x onerror=...&gt; mostrado como texto literal no Impossible (output encoding), sem executar.</t>
+          <t>Entrada #20 — bypasses do High (&amp;, |) bloqueados no Impossible por whitelist de formato IP; resultado sempre idêntico para qualquer input inválido, assinatura de whitelist.</t>
         </is>
       </c>
       <c r="N4" s="5" t="inlineStr">
         <is>
-          <t>⭐⭐</t>
+          <t>⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="O4" s="3" t="inlineStr">
+        <is>
+          <t>Deteção: 🟢 desde a #121 (auditd + regra 100031) — vê a execução de comandos, não o pedido web. Mitigação: nenhuma no lab — o DVWA é vulnerável de propósito (a defesa correta está na coluna "Prevenção" e no nível Impossible).</t>
         </is>
       </c>
     </row>
     <row r="5" ht="110" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>XSS Stored</t>
+          <t>XSS Reflected</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Ataque a aplicações web (injeção de script persistente)</t>
+          <t>Ataque a aplicações web (injeção de script, client-side)</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Script malicioso guardado permanentemente no servidor (comentário, mensagem), executando automaticamente para todos os visitantes da página.</t>
+          <t>Script malicioso refletido de volta na resposta HTTP e executado no browser da vítima; exige que a vítima clique num link preparado.</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Roubo de sessão em massa, desfiguração, redireccionamento para malware, propagação tipo "worm".</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>Alta-Crítica</t>
+          <t>Sequestro de sessão, phishing dentro de um domínio de confiança, entrega de malware.</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Média-Alta</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Confidencialidade, Integridade, Disponibilidade/reputação</t>
+          <t>Confidencialidade (sessão/cookies), Integridade (ações em nome da vítima)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Conteúdo gerado por utilizadores com tags HTML/JS não escapadas na base de dados; comportamento anómalo reportado por múltiplos utilizadores.</t>
+          <t>Parâmetros de URL com tags HTML/JS; violações de CSP registadas; relatos de utilizadores sobre comportamento estranho ao clicar num link.</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Output encoding no momento de apresentar o conteúdo (protege retroativamente até payloads já guardados); sanitização de input; CSP.</t>
+          <t>Output encoding de todo o conteúdo gerado a partir de input do utilizador; Content Security Policy (CSP); cookies HttpOnly.</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>Tipicamente descoberto por relatos externos de utilizadores, não por alerta automático interno; CSP com relatório.</t>
+          <t>WAF; CSP com relatório de violações (report-uri); formação de utilizadores.</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>Remover o payload da base de dados, invalidar sessões, notificar todos os visitantes potencialmente afetados no período de exposição.</t>
+          <t>Invalidar sessões ativas, notificar utilizadores afetados, corrigir o encoding em falta.</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>Output encoding, sanitização de input, CSP, WAF.</t>
+          <t>Output encoding, CSP, HttpOnly, WAF.</t>
         </is>
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>ISO 27001 A.8.28; NIS2 Art.21; RGPD se cookies/dados pessoais de visitantes comprometidos em massa.</t>
+          <t>ISO 27001 A.8.28; NIS2 Art.21.</t>
         </is>
       </c>
       <c r="M5" s="3" t="inlineStr">
         <is>
-          <t>Entrada #28 — payload do nível Low ficou visível como texto ao ser lido através do código Impossible: o encoding acontece na saída, não na gravação.</t>
+          <t>Entrada #24 — payload &lt;img src=x onerror=...&gt; mostrado como texto literal no Impossible (output encoding), sem executar.</t>
         </is>
       </c>
       <c r="N5" s="5" t="inlineStr">
         <is>
-          <t>⭐⭐⭐</t>
+          <t>⭐⭐</t>
+        </is>
+      </c>
+      <c r="O5" s="3" t="inlineStr">
+        <is>
+          <t>Deteção: 🔴. Mitigação: nenhuma no lab — o DVWA é vulnerável de propósito (a defesa correta está na coluna "Prevenção" e no nível Impossible).</t>
         </is>
       </c>
     </row>
     <row r="6" ht="110" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>XSS DOM-based</t>
+          <t>XSS Stored</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Ataque a aplicações web (injeção client-side)</t>
+          <t>Ataque a aplicações web (injeção de script persistente)</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Script malicioso processado inteiramente no browser (JavaScript manipula o DOM a partir de dados não confiáveis, como o URL), sem tocar no servidor.</t>
+          <t>Script malicioso guardado permanentemente no servidor (comentário, mensagem), executando automaticamente para todos os visitantes da página.</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Roubo de sessão, phishing, execução de código no contexto da página.</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>Média-Alta</t>
+          <t>Roubo de sessão em massa, desfiguração, redireccionamento para malware, propagação tipo "worm".</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Alta-Crítica</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Confidencialidade, Integridade</t>
+          <t>Confidencialidade, Integridade, Disponibilidade/reputação</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Nenhum log de servidor regista o ataque; requer monitorização do lado do cliente (RUM, CSP com relatório) para ser visto.</t>
+          <t>Conteúdo gerado por utilizadores com tags HTML/JS não escapadas na base de dados; comportamento anómalo reportado por múltiplos utilizadores.</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>Nunca decodificar/interpretar dados do URL antes de mostrar; usar textContent em vez de innerHTML; CSP.</t>
+          <t>Output encoding no momento de apresentar o conteúdo (protege retroativamente até payloads já guardados); sanitização de input; CSP.</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Tipicamente descoberto externamente (bug bounty, investigador independente) — ponto cego para equipas focadas no servidor.</t>
+          <t>Tipicamente descoberto por relatos externos de utilizadores, não por alerta automático interno; CSP com relatório.</t>
         </is>
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>Corrigir o sink JavaScript inseguro; avaliar prazo de divulgação responsável se reportado externamente.</t>
+          <t>Remover o payload da base de dados, invalidar sessões, notificar todos os visitantes potencialmente afetados no período de exposição.</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>APIs seguras do DOM, CSP com relatório, RUM (Real User Monitoring).</t>
+          <t>Output encoding, sanitização de input, CSP, WAF.</t>
         </is>
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
-          <t>ISO 27001 A.8.28; NIS2 Art.21.</t>
+          <t>ISO 27001 A.8.28; NIS2 Art.21; RGPD se cookies/dados pessoais de visitantes comprometidos em massa.</t>
         </is>
       </c>
       <c r="M6" s="3" t="inlineStr">
         <is>
-          <t>Entrada #32 — valor do URL mostrado codificado (%3Cscript%3E...), nunca decodificado de volta para HTML executável.</t>
+          <t>Entrada #28 — payload do nível Low ficou visível como texto ao ser lido através do código Impossible: o encoding acontece na saída, não na gravação.</t>
         </is>
       </c>
       <c r="N6" s="5" t="inlineStr">
         <is>
-          <t>⭐⭐</t>
+          <t>⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="O6" s="3" t="inlineStr">
+        <is>
+          <t>Deteção: 🔴. Mitigação: nenhuma no lab — o DVWA é vulnerável de propósito (a defesa correta está na coluna "Prevenção" e no nível Impossible).</t>
         </is>
       </c>
     </row>
     <row r="7" ht="110" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>CSRF (Cross-Site Request Forgery)</t>
+          <t>XSS DOM-based</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Ataque a aplicações web (falsificação de pedido entre sites)</t>
+          <t>Ataque a aplicações web (injeção client-side)</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Força a vítima autenticada a executar uma ação não intencional (ex. mudar password) através de um pedido forjado noutra página, sem roubar credenciais.</t>
+          <t>Script malicioso processado inteiramente no browser (JavaScript manipula o DOM a partir de dados não confiáveis, como o URL), sem tocar no servidor.</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Executar ações autorizadas da vítima sem o seu conhecimento (mudar password, transferir fundos, alterar permissões).</t>
+          <t>Roubo de sessão, phishing, execução de código no contexto da página.</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Média-Alta</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Integridade (ações não autorizadas); Confidencialidade/Disponibilidade dependendo da ação forjada</t>
+          <t>Confidencialidade, Integridade</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>Pedidos sem token CSRF válido; ausência de cabeçalho Referer/Origin esperado; mudanças de conta não iniciadas pelo utilizador.</t>
+          <t>Nenhum log de servidor regista o ataque; requer monitorização do lado do cliente (RUM, CSP com relatório) para ser visto.</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>Tokens anti-CSRF únicos por sessão/pedido; verificar a password atual em ações sensíveis; cookies SameSite.</t>
+          <t>Nunca decodificar/interpretar dados do URL antes de mostrar; usar textContent em vez de innerHTML; CSP.</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Monitorização de pedidos sem token válido; alertas de mudança de conta fora do padrão de navegação normal.</t>
+          <t>Tipicamente descoberto externamente (bug bounty, investigador independente) — ponto cego para equipas focadas no servidor.</t>
         </is>
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>Reverter a ação forjada, forçar novo login, verificar se há mais contas afetadas pela mesma campanha.</t>
+          <t>Corrigir o sink JavaScript inseguro; avaliar prazo de divulgação responsável se reportado externamente.</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>Tokens anti-CSRF, cookies SameSite, confirmação de password em ações sensíveis.</t>
+          <t>APIs seguras do DOM, CSP com relatório, RUM (Real User Monitoring).</t>
         </is>
       </c>
       <c r="L7" s="3" t="inlineStr">
@@ -1012,69 +978,74 @@
       </c>
       <c r="M7" s="3" t="inlineStr">
         <is>
-          <t>Entrada #36 — tag &lt;img&gt; a apontar para o URL de mudança de password, bloqueada no Impossible por token anti-CSRF (só passou por um falso positivo de ambiente contaminado, corrigido antes de confirmar).</t>
+          <t>Entrada #32 — valor do URL mostrado codificado (%3Cscript%3E...), nunca decodificado de volta para HTML executável.</t>
         </is>
       </c>
       <c r="N7" s="5" t="inlineStr">
         <is>
           <t>⭐⭐</t>
+        </is>
+      </c>
+      <c r="O7" s="3" t="inlineStr">
+        <is>
+          <t>Deteção: 🔴. Mitigação: nenhuma no lab — o DVWA é vulnerável de propósito (a defesa correta está na coluna "Prevenção" e no nível Impossible).</t>
         </is>
       </c>
     </row>
     <row r="8" ht="110" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>File Upload malicioso</t>
+          <t>CSRF (Cross-Site Request Forgery)</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Ataque a aplicações web (upload de ficheiro malicioso)</t>
+          <t>Ataque a aplicações web (falsificação de pedido entre sites)</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Envio de um ficheiro executável (ex. web shell PHP) disfarçado ou aceite sem validação suficiente, ficando disponível para execução no servidor.</t>
+          <t>Força a vítima autenticada a executar uma ação não intencional (ex. mudar password) através de um pedido forjado noutra página, sem roubar credenciais.</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Execução remota de código (RCE); acesso persistente ao servidor via web shell.</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>Crítica</t>
+          <t>Executar ações autorizadas da vítima sem o seu conhecimento (mudar password, transferir fundos, alterar permissões).</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>Alta</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Confidencialidade, Integridade, Disponibilidade</t>
+          <t>Integridade (ações não autorizadas); Confidencialidade/Disponibilidade dependendo da ação forjada</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>Ficheiros com extensões executáveis em pastas de upload; discrepância entre Content-Type declarado e conteúdo real; pedidos a ficheiros recém-carregados com parâmetros tipo ?cmd=.</t>
+          <t>Pedidos sem token CSRF válido; ausência de cabeçalho Referer/Origin esperado; mudanças de conta não iniciadas pelo utilizador.</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>Validação real do conteúdo do ficheiro (nunca só extensão/MIME type); desativar execução de scripts em pastas de upload; token anti-CSRF no formulário.</t>
+          <t>Tokens anti-CSRF únicos por sessão/pedido; verificar a password atual em ações sensíveis; cookies SameSite.</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Scanners de integridade de ficheiros (FIM); antivírus nas pastas de upload; alertas de novos ficheiros executáveis.</t>
+          <t>Monitorização de pedidos sem token válido; alertas de mudança de conta fora do padrão de navegação normal.</t>
         </is>
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>Localizar e remover TODOS os web shells (corrigir a validação não remove os já colocados); rever logs para identificar o alcance do acesso obtido.</t>
+          <t>Reverter a ação forjada, forçar novo login, verificar se há mais contas afetadas pela mesma campanha.</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>FIM (File Integrity Monitoring), antivírus/EDR, isolamento da pasta de upload sem permissão de execução, CDN/storage externo.</t>
+          <t>Tokens anti-CSRF, cookies SameSite, confirmação de password em ações sensíveis.</t>
         </is>
       </c>
       <c r="L8" s="3" t="inlineStr">
@@ -1084,69 +1055,74 @@
       </c>
       <c r="M8" s="3" t="inlineStr">
         <is>
-          <t>Entrada #40 — shell.php aceite sem validação no Low/Medium; bloqueado no High/Impossible por validação de tipo + token anti-CSRF.</t>
+          <t>Entrada #36 — tag &lt;img&gt; a apontar para o URL de mudança de password, bloqueada no Impossible por token anti-CSRF (só passou por um falso positivo de ambiente contaminado, corrigido antes de confirmar).</t>
         </is>
       </c>
       <c r="N8" s="5" t="inlineStr">
         <is>
-          <t>⭐⭐⭐</t>
+          <t>⭐⭐</t>
+        </is>
+      </c>
+      <c r="O8" s="3" t="inlineStr">
+        <is>
+          <t>Deteção: 🔴. Mitigação: nenhuma no lab — o DVWA é vulnerável de propósito (a defesa correta está na coluna "Prevenção" e no nível Impossible).</t>
         </is>
       </c>
     </row>
     <row r="9" ht="110" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>File Inclusion (LFI/RFI)</t>
+          <t>File Upload malicioso</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Ataque a aplicações web (inclusão de ficheiros local/remota)</t>
+          <t>Ataque a aplicações web (upload de ficheiro malicioso)</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Manipulação de um parâmetro que controla qual ficheiro o servidor inclui/executa, permitindo ler ficheiros locais sensíveis (LFI) ou, com allow_url_include ativo, executar código remoto (RFI).</t>
+          <t>Envio de um ficheiro executável (ex. web shell PHP) disfarçado ou aceite sem validação suficiente, ficando disponível para execução no servidor.</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Exposição de ficheiros de configuração/credenciais (LFI); execução remota de código (RFI).</t>
+          <t>Execução remota de código (RCE); acesso persistente ao servidor via web shell.</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Alta a Crítica</t>
+          <t>Crítica</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Confidencialidade (LFI); + Integridade/Disponibilidade se encadeado com RFI ou upload</t>
+          <t>Confidencialidade, Integridade, Disponibilidade</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Parâmetros de página com caminhos de ficheiro (../, file://, URLs externos); pedidos a /etc/passwd ou ficheiros de configuração.</t>
+          <t>Ficheiros com extensões executáveis em pastas de upload; discrepância entre Content-Type declarado e conteúdo real; pedidos a ficheiros recém-carregados com parâmetros tipo ?cmd=.</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>Whitelist exata de valores permitidos (nunca verificação de prefixo/padrão); desativar allow_url_include no PHP; nunca usar input do utilizador diretamente numa chamada de inclusão.</t>
+          <t>Validação real do conteúdo do ficheiro (nunca só extensão/MIME type); desativar execução de scripts em pastas de upload; token anti-CSRF no formulário.</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>WAF; alertas de acesso a ficheiros de sistema fora do webroot.</t>
+          <t>Scanners de integridade de ficheiros (FIM); antivírus nas pastas de upload; alertas de novos ficheiros executáveis.</t>
         </is>
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>Rever quais credenciais/ficheiros de configuração foram expostos e rodá-las; corrigir a whitelist.</t>
+          <t>Localizar e remover TODOS os web shells (corrigir a validação não remove os já colocados); rever logs para identificar o alcance do acesso obtido.</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>Whitelist exata, configuração segura do PHP (allow_url_include Off), WAF.</t>
+          <t>FIM (File Integrity Monitoring), antivírus/EDR, isolamento da pasta de upload sem permissão de execução, CDN/storage externo.</t>
         </is>
       </c>
       <c r="L9" s="3" t="inlineStr">
@@ -1156,399 +1132,429 @@
       </c>
       <c r="M9" s="3" t="inlineStr">
         <is>
-          <t>Entrada #44 — bypass file:// do High (verificação de prefixo) bloqueado no Impossible por whitelist exata (comparação por igualdade, não por prefixo).</t>
+          <t>Entrada #40 — shell.php aceite sem validação no Low/Medium; bloqueado no High/Impossible por validação de tipo + token anti-CSRF.</t>
         </is>
       </c>
       <c r="N9" s="5" t="inlineStr">
         <is>
-          <t>⭐⭐</t>
+          <t>⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="O9" s="3" t="inlineStr">
+        <is>
+          <t>Deteção: 🔴 (a regra 100031 da #121 pode ver a execução posterior, mas esta cadeia não foi retestada). Mitigação: nenhuma no lab — o DVWA é vulnerável de propósito (a defesa correta está na coluna "Prevenção" e no nível Impossible).</t>
         </is>
       </c>
     </row>
     <row r="10" ht="110" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>RCE encadeado (File Upload + File Inclusion)</t>
+          <t>File Inclusion (LFI/RFI)</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Ataque a aplicações web (encadeamento de vulnerabilidades)</t>
+          <t>Ataque a aplicações web (inclusão de ficheiros local/remota)</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Combinação de duas funcionalidades individualmente "seguras" — upload de uma imagem genuinamente válida com payload PHP escondido, seguida de inclusão desse ficheiro por outra funcionalidade — resultando em execução de código.</t>
+          <t>Manipulação de um parâmetro que controla qual ficheiro o servidor inclui/executa, permitindo ler ficheiros locais sensíveis (LFI) ou, com allow_url_include ativo, executar código remoto (RFI).</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Execução remota de código, contornando as defesas de cada funcionalidade avaliada isoladamente.</t>
+          <t>Exposição de ficheiros de configuração/credenciais (LFI); execução remota de código (RFI).</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Crítica</t>
+          <t>Alta a Crítica</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>Confidencialidade, Integridade, Disponibilidade</t>
+          <t>Confidencialidade (LFI); + Integridade/Disponibilidade se encadeado com RFI ou upload</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>Nenhum sinal isolado óbvio — a imagem passa scanners de malware normalmente; só a correlação entre o upload e o pedido de inclusão posterior revela o ataque.</t>
+          <t>Parâmetros de página com caminhos de ficheiro (../, file://, URLs externos); pedidos a /etc/passwd ou ficheiros de configuração.</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>Defesa em profundidade: travar qualquer elo da cadeia (validação de upload OU whitelist de inclusão) já é suficiente; nunca avaliar funcionalidades isoladamente numa auditoria.</t>
+          <t>Whitelist exata de valores permitidos (nunca verificação de prefixo/padrão); desativar allow_url_include no PHP; nunca usar input do utilizador diretamente numa chamada de inclusão.</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Correlação entre eventos de upload e de inclusão/leitura de ficheiro (SIEM); scanners de malware não bastam, o ficheiro é uma imagem válida.</t>
+          <t>WAF; alertas de acesso a ficheiros de sistema fora do webroot.</t>
         </is>
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>Identificar todos os ficheiros "imagem" com payload embutido já carregados; corrigir o elo mais fraco da cadeia.</t>
+          <t>Rever quais credenciais/ficheiros de configuração foram expostos e rodá-las; corrigir a whitelist.</t>
         </is>
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>Whitelist exata de inclusão, validação de conteúdo real do ficheiro, SIEM com correlação entre funcionalidades.</t>
+          <t>Whitelist exata, configuração segura do PHP (allow_url_include Off), WAF.</t>
         </is>
       </c>
       <c r="L10" s="3" t="inlineStr">
         <is>
-          <t>ISO 27001 A.8.28, A.8.29 (testes de segurança); NIS2 Art.21.</t>
+          <t>ISO 27001 A.8.28; NIS2 Art.21.</t>
         </is>
       </c>
       <c r="M10" s="3" t="inlineStr">
         <is>
-          <t>Entradas #45/#46 — polyglot.jpg com payload PHP, executável via File Inclusion no nível High mas bloqueado no Impossible pela whitelist exata.</t>
+          <t>Entrada #44 — bypass file:// do High (verificação de prefixo) bloqueado no Impossible por whitelist exata (comparação por igualdade, não por prefixo).</t>
         </is>
       </c>
       <c r="N10" s="5" t="inlineStr">
         <is>
           <t>⭐⭐</t>
+        </is>
+      </c>
+      <c r="O10" s="3" t="inlineStr">
+        <is>
+          <t>Deteção: 🔴. Mitigação: nenhuma no lab — o DVWA é vulnerável de propósito (a defesa correta está na coluna "Prevenção" e no nível Impossible).</t>
         </is>
       </c>
     </row>
     <row r="11" ht="110" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Brute Force (credenciais)</t>
+          <t>RCE encadeado (File Upload + File Inclusion)</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Ataque a credenciais</t>
+          <t>Ataque a aplicações web (encadeamento de vulnerabilidades)</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Tentativas repetidas e automatizadas de adivinhar uma password através de uma wordlist, contra um único utilizador-alvo.</t>
+          <t>Combinação de duas funcionalidades individualmente "seguras" — upload de uma imagem genuinamente válida com payload PHP escondido, seguida de inclusão desse ficheiro por outra funcionalidade — resultando em execução de código.</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Obter acesso a uma conta específica adivinhando a password.</t>
-        </is>
-      </c>
-      <c r="E11" s="6" t="inlineStr">
-        <is>
-          <t>Média-Alta</t>
+          <t>Execução remota de código, contornando as defesas de cada funcionalidade avaliada isoladamente.</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Crítica</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Confidencialidade, Integridade</t>
+          <t>Confidencialidade, Integridade, Disponibilidade</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>Múltiplas tentativas de login falhadas na mesma conta num curto espaço de tempo; padrão de tentativas sequenciais tipo dicionário.</t>
+          <t>Nenhum sinal isolado óbvio — a imagem passa scanners de malware normalmente; só a correlação entre o upload e o pedido de inclusão posterior revela o ataque.</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>Bloqueio de conta / rate limiting após N falhas (ataca o volume de tentativas, não só o custo); MFA; prepared statements no próprio formulário de login.</t>
+          <t>Defesa em profundidade: travar qualquer elo da cadeia (validação de upload OU whitelist de inclusão) já é suficiente; nunca avaliar funcionalidades isoladamente numa auditoria.</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>Alertas de múltiplas falhas de autenticação na mesma conta/IP num curto período.</t>
+          <t>Correlação entre eventos de upload e de inclusão/leitura de ficheiro (SIEM); scanners de malware não bastam, o ficheiro é uma imagem válida.</t>
         </is>
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>Confirmar se a conta foi comprometida antes do bloqueio; forçar reset de password; verificar se há tentativas distribuídas (credential stuffing associado).</t>
+          <t>Identificar todos os ficheiros "imagem" com payload embutido já carregados; corrigir o elo mais fraco da cadeia.</t>
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>Account lockout, rate limiting, MFA, CAPTCHA.</t>
+          <t>Whitelist exata de inclusão, validação de conteúdo real do ficheiro, SIEM com correlação entre funcionalidades.</t>
         </is>
       </c>
       <c r="L11" s="3" t="inlineStr">
         <is>
-          <t>ISO 27001 A.5.17 (gestão de direitos de acesso), A.8.28; NIS2 Art.21.</t>
+          <t>ISO 27001 A.8.28, A.8.29 (testes de segurança); NIS2 Art.21.</t>
         </is>
       </c>
       <c r="M11" s="3" t="inlineStr">
         <is>
-          <t>Entrada #51 — password correta na wordlist em 5º lugar, mas bloqueio de conta ao fim de 3 falhas neutralizou o ataque no Impossible antes de lá chegar.</t>
+          <t>Entradas #45/#46 — polyglot.jpg com payload PHP, executável via File Inclusion no nível High mas bloqueado no Impossible pela whitelist exata.</t>
         </is>
       </c>
       <c r="N11" s="5" t="inlineStr">
         <is>
-          <t>⭐⭐⭐</t>
+          <t>⭐⭐</t>
+        </is>
+      </c>
+      <c r="O11" s="3" t="inlineStr">
+        <is>
+          <t>Deteção: 🔴 (mesma nota da linha 7, não retestado). Mitigação: nenhuma no lab — o DVWA é vulnerável de propósito (a defesa correta está na coluna "Prevenção" e no nível Impossible).</t>
         </is>
       </c>
     </row>
     <row r="12" ht="110" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>FTP anónimo + Apache = RCE (cadeia de serviços)</t>
+          <t>Brute Force (credenciais)</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Ataque à rede (cadeia de má configuração de serviços)</t>
+          <t>Ataque a credenciais</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Escrita anónima permitida num serviço FTP combinada com um servidor web a servir a mesma pasta, permitindo carregar e depois executar um web shell PHP sem qualquer credencial.</t>
+          <t>Tentativas repetidas e automatizadas de adivinhar uma password através de uma wordlist, contra um único utilizador-alvo.</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Execução remota de código através do encadeamento de dois serviços mal configurados.</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>Crítica</t>
+          <t>Obter acesso a uma conta específica adivinhando a password.</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>Média-Alta</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Confidencialidade, Integridade, Disponibilidade</t>
+          <t>Confidencialidade, Integridade</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>Acesso FTP anónimo com permissão de escrita; DocumentRoot do servidor web a coincidir com pasta de upload de outro serviço; pedidos HTTP a ficheiros .php recém-criados.</t>
+          <t>Múltiplas tentativas de login falhadas na mesma conta num curto espaço de tempo; padrão de tentativas sequenciais tipo dicionário.</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>Nunca ativar escrita anónima em FTP; nunca fazer coincidir a pasta do FTP com a pasta servida pela web; desativar execução de scripts em pastas de upload.</t>
+          <t>Bloqueio de conta / rate limiting após N falhas (ataca o volume de tentativas, não só o custo); MFA; prepared statements no próprio formulário de login.</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>Correlação entre logs de FTP e logs do servidor web — sem um SIEM, a ligação entre os dois eventos passa despercebida.</t>
+          <t>Alertas de múltiplas falhas de autenticação na mesma conta/IP num curto período.</t>
         </is>
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>Localizar e remover web shells; desativar escrita anónima; segmentar pastas de upload das pastas servidas.</t>
+          <t>Confirmar se a conta foi comprometida antes do bloqueio; forçar reset de password; verificar se há tentativas distribuídas (credential stuffing associado).</t>
         </is>
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>SIEM (correlação entre serviços), segmentação de pastas, desativação de execução de scripts em uploads.</t>
+          <t>Account lockout, rate limiting, MFA, CAPTCHA.</t>
         </is>
       </c>
       <c r="L12" s="3" t="inlineStr">
         <is>
-          <t>ISO 27001 A.8.9 (gestão de configuração), A.8.16 (monitorização); NIS2 Art.21.</t>
+          <t>ISO 27001 A.5.17 (gestão de direitos de acesso), A.8.28; NIS2 Art.21.</t>
         </is>
       </c>
       <c r="M12" s="3" t="inlineStr">
         <is>
-          <t>Entrada #60 — shell.php enviado por FTP anónimo, executado via curl no Apache (porta 8080), devolvendo www-data.</t>
+          <t>Entrada #51 — password correta na wordlist em 5º lugar, mas bloqueio de conta ao fim de 3 falhas neutralizou o ataque no Impossible antes de lá chegar.</t>
         </is>
       </c>
       <c r="N12" s="5" t="inlineStr">
         <is>
-          <t>⭐⭐</t>
+          <t>⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="O12" s="3" t="inlineStr">
+        <is>
+          <t>Deteção: 🔴 no DVWA. Mitigação: no domínio, bloqueio de conta (Fase 5) e política de 16 caracteres (Fase 8); no DVWA, só no nível Impossible.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="110" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Optionsbleed (CVE-2017-9798)</t>
+          <t>FTP anónimo + Apache = RCE (cadeia de serviços)</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Vulnerabilidade de software (divulgação de memória)</t>
+          <t>Ataque à rede (cadeia de má configuração de serviços)</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Falha em versões antigas do Apache (&lt; 2.4.27) que, sob configuração .htaccess específica (diretivas Limit/LimitExcept contraditórias), pode divulgar memória do processo no cabeçalho Allow.</t>
+          <t>Escrita anónima permitida num serviço FTP combinada com um servidor web a servir a mesma pasta, permitindo carregar e depois executar um web shell PHP sem qualquer credencial.</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Divulgação de memória do processo (potencialmente credenciais ou tokens de sessão de outros pedidos concorrentes).</t>
-        </is>
-      </c>
-      <c r="E13" s="7" t="inlineStr">
-        <is>
-          <t>Média (teórica; depende de configuração muito específica para ser explorável)</t>
+          <t>Execução remota de código através do encadeamento de dois serviços mal configurados.</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Crítica</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Confidencialidade</t>
+          <t>Confidencialidade, Integridade, Disponibilidade</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>Cabeçalho Allow inconsistente ou corrompido em respostas a pedidos OPTIONS; versão de Apache no intervalo afetado.</t>
+          <t>Acesso FTP anónimo com permissão de escrita; DocumentRoot do servidor web a coincidir com pasta de upload de outro serviço; pedidos HTTP a ficheiros .php recém-criados.</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>Atualizar Apache para versão ≥ 2.4.27; rever ficheiros .htaccess com diretivas Limit/LimitExcept contraditórias.</t>
+          <t>Nunca ativar escrita anónima em FTP; nunca fazer coincidir a pasta do FTP com a pasta servida pela web; desativar execução de scripts em pastas de upload.</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>Scanner de vulnerabilidades a assinalar a versão; teste ativo com múltiplos pedidos OPTIONS concorrentes para confirmar exploração real.</t>
+          <t>Correlação entre logs de FTP e logs do servidor web — sem um SIEM, a ligação entre os dois eventos passa despercebida.</t>
         </is>
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>Atualizar o software; se confirmado explorado, assumir possível exposição de dados de outros pedidos concorrentes.</t>
+          <t>Localizar e remover web shells; desativar escrita anónima; segmentar pastas de upload das pastas servidas.</t>
         </is>
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>Gestão de patches, scanners de vulnerabilidades com triagem manual.</t>
+          <t>SIEM (correlação entre serviços), segmentação de pastas, desativação de execução de scripts em uploads.</t>
         </is>
       </c>
       <c r="L13" s="3" t="inlineStr">
         <is>
-          <t>ISO 27001 A.8.8 (gestão de vulnerabilidades técnicas); NIS2 Art.21; risco aceite formal exigido mesmo sem exploração confirmada (ex. ISO 27001/PCI-DSS).</t>
+          <t>ISO 27001 A.8.9 (gestão de configuração), A.8.16 (monitorização); NIS2 Art.21.</t>
         </is>
       </c>
       <c r="M13" s="3" t="inlineStr">
         <is>
-          <t>Entrada #62 — versão de Apache no intervalo afetado, mas vulnerabilidade não reproduzida mesmo sob 50 pedidos OPTIONS simultâneos; resultado negativo documentado formalmente, não ignorado.</t>
+          <t>Entrada #60 — shell.php enviado por FTP anónimo, executado via curl no Apache (porta 8080), devolvendo www-data.</t>
         </is>
       </c>
       <c r="N13" s="5" t="inlineStr">
         <is>
-          <t>⭐</t>
+          <t>⭐⭐</t>
+        </is>
+      </c>
+      <c r="O13" s="3" t="inlineStr">
+        <is>
+          <t>Deteção: 🟢 desde a #102. Mitigação: causa corrigida na #104 (FTP só de leitura, PHP desligado na pasta de upload); recusa reconfirmada ao vivo a 2026-10-19 (#129). Por tratar na Fase 10: pasta de upload a 777 e caminhos de escrita anónima (risco #1).</t>
         </is>
       </c>
     </row>
     <row r="14" ht="110" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Samba — partilha anónima mal configurada</t>
+          <t>Optionsbleed (CVE-2017-9798)</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Ataque à rede (má configuração de partilha de ficheiros)</t>
+          <t>Vulnerabilidade de software (divulgação de memória)</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Partilha de rede Samba configurada para aceitar ligações anónimas (guest ok) com permissão de escrita, permitindo enumeração e upload de ficheiros sem qualquer credencial.</t>
+          <t>Falha em versões antigas do Apache (&lt; 2.4.27) que, sob configuração .htaccess específica (diretivas Limit/LimitExcept contraditórias), pode divulgar memória do processo no cabeçalho Allow.</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Acesso não autorizado a ficheiros partilhados; ponto de apoio para distribuir malware/ransomware pela rede.</t>
-        </is>
-      </c>
-      <c r="E14" s="6" t="inlineStr">
-        <is>
-          <t>Alta</t>
+          <t>Divulgação de memória do processo (potencialmente credenciais ou tokens de sessão de outros pedidos concorrentes).</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Média (teórica; depende de configuração muito específica para ser explorável)</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Confidencialidade, Integridade, Disponibilidade</t>
+          <t>Confidencialidade</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>Partilhas visíveis sem autenticação (smbclient -L // -N); escrita bem-sucedida sem credenciais.</t>
+          <t>Cabeçalho Allow inconsistente ou corrompido em respostas a pedidos OPTIONS; versão de Apache no intervalo afetado.</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>Nunca ativar guest ok = yes salvo necessidade real; restringir sempre escrita quando o acesso anónimo for necessário; segmentar as portas SMB (139/445).</t>
+          <t>Atualizar Apache para versão ≥ 2.4.27; rever ficheiros .htaccess com diretivas Limit/LimitExcept contraditórias.</t>
         </is>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>Auditoria periódica de configuração de partilhas; monitorização de acessos SMB anónimos.</t>
+          <t>Scanner de vulnerabilidades a assinalar a versão; teste ativo com múltiplos pedidos OPTIONS concorrentes para confirmar exploração real.</t>
         </is>
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
-          <t>Desativar o acesso anónimo; rever ficheiros colocados na partilha; verificar sinais de propagação lateral.</t>
+          <t>Atualizar o software; se confirmado explorado, assumir possível exposição de dados de outros pedidos concorrentes.</t>
         </is>
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>Segmentação de rede, auditoria de configuração, princípio do menor privilégio em partilhas.</t>
+          <t>Gestão de patches, scanners de vulnerabilidades com triagem manual.</t>
         </is>
       </c>
       <c r="L14" s="3" t="inlineStr">
         <is>
-          <t>ISO 27001 A.8.3 (restrição de acesso à informação), A.8.20 (segurança de redes); NIS2 Art.21.</t>
+          <t>ISO 27001 A.8.8 (gestão de vulnerabilidades técnicas); NIS2 Art.21; risco aceite formal exigido mesmo sem exploração confirmada (ex. ISO 27001/PCI-DSS).</t>
         </is>
       </c>
       <c r="M14" s="3" t="inlineStr">
         <is>
-          <t>Entrada #64 — partilha publico com guest ok=yes e read only=no, enumerada e escrita a partir do Kali sem qualquer credencial.</t>
+          <t>Entrada #62 — versão de Apache no intervalo afetado, mas vulnerabilidade não reproduzida mesmo sob 50 pedidos OPTIONS simultâneos; resultado negativo documentado formalmente, não ignorado.</t>
         </is>
       </c>
       <c r="N14" s="5" t="inlineStr">
         <is>
-          <t>⭐⭐</t>
+          <t>⭐</t>
+        </is>
+      </c>
+      <c r="O14" s="3" t="inlineStr">
+        <is>
+          <t>Deteção: 🔴 (sondagem). Mitigação: nenhuma — patches em risco aceite (#6); vulnerabilidade não reproduzida (#62); versão antiga confirmada pelo scanner (#126).</t>
         </is>
       </c>
     </row>
     <row r="15" ht="110" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>MariaDB — credenciais fracas e sem cifra</t>
+          <t>Samba — partilha anónima mal configurada</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Ataque a credenciais (base de dados exposta)</t>
+          <t>Ataque à rede (má configuração de partilha de ficheiros)</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Base de dados exposta à rede com bind-address aberto, credenciais fracas/por defeito e sem cifra de ligação (TLS).</t>
+          <t>Partilha de rede Samba configurada para aceitar ligações anónimas (guest ok) com permissão de escrita, permitindo enumeração e upload de ficheiros sem qualquer credencial.</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Acesso não autorizado à base de dados completa.</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>Crítica</t>
+          <t>Acesso não autorizado a ficheiros partilhados; ponto de apoio para distribuir malware/ransomware pela rede.</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>Alta</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
@@ -1558,265 +1564,285 @@
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>Porta de base de dados (3306) acessível fora do localhost; tentativas de login com utilizadores comuns (root, admin); ligações sem TLS.</t>
+          <t>Partilhas visíveis sem autenticação (smbclient -L // -N); escrita bem-sucedida sem credenciais.</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>bind-address = 127.0.0.1 por defeito; passwords fortes; restringir por IP de origem; ativar TLS no servidor de base de dados.</t>
+          <t>Nunca ativar guest ok = yes salvo necessidade real; restringir sempre escrita quando o acesso anónimo for necessário; segmentar as portas SMB (139/445).</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>Monitorização de logins na BD a partir de IPs não esperados; scanner de portas expostas.</t>
+          <t>Auditoria periódica de configuração de partilhas; monitorização de acessos SMB anónimos.</t>
         </is>
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t>Rodar credenciais, restringir o acesso de rede, ativar TLS, auditar que dados foram acedidos/alterados.</t>
+          <t>Desativar o acesso anónimo; rever ficheiros colocados na partilha; verificar sinais de propagação lateral.</t>
         </is>
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>Firewall/segmentação de rede, TLS em bases de dados, gestão de credenciais/cofre de segredos.</t>
+          <t>Segmentação de rede, auditoria de configuração, princípio do menor privilégio em partilhas.</t>
         </is>
       </c>
       <c r="L15" s="3" t="inlineStr">
         <is>
-          <t>ISO 27001 A.8.24 (criptografia), A.8.20; NIS2 Art.21; PCI-DSS (cifra em trânsito obrigatória para dados de pagamento); RGPD se dados pessoais na BD.</t>
+          <t>ISO 27001 A.8.3 (restrição de acesso à informação), A.8.20 (segurança de redes); NIS2 Art.21.</t>
         </is>
       </c>
       <c r="M15" s="3" t="inlineStr">
         <is>
-          <t>Entrada #65 — utilizador dbadmin/admin123, acesso total confirmado manualmente e via Metasploit, sem TLS.</t>
+          <t>Entrada #64 — partilha publico com guest ok=yes e read only=no, enumerada e escrita a partir do Kali sem qualquer credencial.</t>
         </is>
       </c>
       <c r="N15" s="5" t="inlineStr">
         <is>
-          <t>⭐⭐⭐</t>
+          <t>⭐⭐</t>
+        </is>
+      </c>
+      <c r="O15" s="3" t="inlineStr">
+        <is>
+          <t>Deteção: 🔴. Mitigação: por verificar — escrita anónima não reverificada desde a #64 (exposição confirmada na #126); verificação na Fase 10.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="110" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Enumeração de Active Directory sem credenciais</t>
+          <t>MariaDB — credenciais fracas e sem cifra</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Ataque à rede (reconhecimento, Active Directory)</t>
+          <t>Ataque a credenciais (base de dados exposta)</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Recolha de informação sobre um domínio Active Directory (nmap, scripts LDAP/SMB, bind anónimo, transferência de zona DNS) sem qualquer credencial válida — vista de atacante externo.</t>
+          <t>Base de dados exposta à rede com bind-address aberto, credenciais fracas/por defeito e sem cifra de ligação (TLS).</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Mapear a superfície do domínio antes de decidir por onde tentar entrar (reconhecimento pré-ataque).</t>
-        </is>
-      </c>
-      <c r="E16" s="8" t="inlineStr">
-        <is>
-          <t>Baixa isolada (alimenta ataques posteriores mais graves)</t>
+          <t>Acesso não autorizado à base de dados completa.</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Crítica</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Confidencialidade (informação de reconhecimento)</t>
+          <t>Confidencialidade, Integridade, Disponibilidade</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>Isolado, indistinguível de tráfego legítimo; só a correlação de sequência (scan de portas + LDAP + sessão SMB nula + tentativa de transferência de zona, do mesmo IP, em pouco tempo) revela reconhecimento real.</t>
+          <t>Porta de base de dados (3306) acessível fora do localhost; tentativas de login com utilizadores comuns (root, admin); ligações sem TLS.</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>Desativar bind LDAP anónimo; RestrictAnonymous a nível 1-2; restringir transferência de zona DNS; manter SMB signing ativo.</t>
+          <t>bind-address = 127.0.0.1 por defeito; passwords fortes; restringir por IP de origem; ativar TLS no servidor de base de dados.</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>Correlação de eventos entre múltiplos protocolos num SIEM — deteção isolada por evento gera demasiados falsos positivos.</t>
+          <t>Monitorização de logins na BD a partir de IPs não esperados; scanner de portas expostas.</t>
         </is>
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
-          <t>Identificar e bloquear o IP de origem; reforçar os controlos que ainda estejam mal configurados.</t>
+          <t>Rodar credenciais, restringir o acesso de rede, ativar TLS, auditar que dados foram acedidos/alterados.</t>
         </is>
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>SIEM com correlação, hardening de LDAP/SMB/DNS, IDS/IPS.</t>
+          <t>Firewall/segmentação de rede, TLS em bases de dados, gestão de credenciais/cofre de segredos.</t>
         </is>
       </c>
       <c r="L16" s="3" t="inlineStr">
         <is>
-          <t>ISO 27001 A.8.16 (monitorização de atividades); NIS2 Art.21; MITRE ATT&amp;CK T1087/T1018.</t>
+          <t>ISO 27001 A.8.24 (criptografia), A.8.20; NIS2 Art.21; PCI-DSS (cifra em trânsito obrigatória para dados de pagamento); RGPD se dados pessoais na BD.</t>
         </is>
       </c>
       <c r="M16" s="3" t="inlineStr">
         <is>
-          <t>Entrada #89 — RootDSE do LDAP exposto por definição de protocolo (não é falha); bind anónimo, listagem SMB e transferência de zona corretamente bloqueados neste domínio.</t>
+          <t>Entrada #65 — utilizador dbadmin/admin123, acesso total confirmado manualmente e via Metasploit, sem TLS.</t>
         </is>
       </c>
       <c r="N16" s="5" t="inlineStr">
         <is>
           <t>⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="O16" s="3" t="inlineStr">
+        <is>
+          <t>Deteção: 🟡 (o dado existe, sem alerta dedicado). Mitigação: nenhuma — exposição mantida como material de exercício (#126).</t>
         </is>
       </c>
     </row>
     <row r="17" ht="110" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>BloodHound — mapeamento de caminhos de ataque em AD</t>
+          <t>Enumeração de Active Directory sem credenciais</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Ataque à rede (reconhecimento autenticado / escalação de privilégios, Active Directory)</t>
+          <t>Ataque à rede (reconhecimento, Active Directory)</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Recolha e visualização gráfica das relações de permissões do Active Directory para identificar caminhos possíveis de escalação de privilégio até Domain Admin, a partir de uma conta de baixo privilégio.</t>
+          <t>Recolha de informação sobre um domínio Active Directory (nmap, scripts LDAP/SMB, bind anónimo, transferência de zona DNS) sem qualquer credencial válida — vista de atacante externo.</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Encontrar um caminho de escalação de privilégio vertical dentro do domínio.</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>Crítica se existir caminho; informativa se não existir</t>
+          <t>Mapear a superfície do domínio antes de decidir por onde tentar entrar (reconhecimento pré-ataque).</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>Baixa isolada (alimenta ataques posteriores mais graves)</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Confidencialidade, Integridade, Disponibilidade (compromisso total do domínio se o caminho existir e for explorado)</t>
+          <t>Confidencialidade (informação de reconhecimento)</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>Volume anómalo de consultas LDAP/SMB de uma única conta num curto espaço de tempo — assinatura típica de um collector (SharpHound/bloodhound-python).</t>
+          <t>Isolado, indistinguível de tráfego legítimo; só a correlação de sequência (scan de portas + LDAP + sessão SMB nula + tentativa de transferência de zona, do mesmo IP, em pouco tempo) revela reconhecimento real.</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>Princípio do menor privilégio consistente; rever e reverter permissões temporárias; auditorias BloodHound próprias e periódicas (uso defensivo da mesma ferramenta).</t>
+          <t>Desativar bind LDAP anónimo; RestrictAnonymous a nível 1-2; restringir transferência de zona DNS; manter SMB signing ativo.</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>Monitorização de volume de consultas LDAP de uma única conta; Microsoft Defender for Identity ou equivalente.</t>
+          <t>Correlação de eventos entre múltiplos protocolos num SIEM — deteção isolada por evento gera demasiados falsos positivos.</t>
         </is>
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
-          <t>Se um caminho for encontrado, corrigir a cadeia de permissões que o permite, não só o nó final.</t>
+          <t>Identificar e bloquear o IP de origem; reforçar os controlos que ainda estejam mal configurados.</t>
         </is>
       </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t>Auditoria periódica com BloodHound (defensiva), Defender for Identity, revisão de grupos privilegiados.</t>
+          <t>SIEM com correlação, hardening de LDAP/SMB/DNS, IDS/IPS.</t>
         </is>
       </c>
       <c r="L17" s="3" t="inlineStr">
         <is>
-          <t>ISO 27001 A.5.15 (controlo de acesso), A.8.2 (direitos de acesso privilegiado); NIS2 Art.21; MITRE ATT&amp;CK T1087/T1069/T1482.</t>
+          <t>ISO 27001 A.8.16 (monitorização de atividades); NIS2 Art.21; MITRE ATT&amp;CK T1087/T1018.</t>
         </is>
       </c>
       <c r="M17" s="3" t="inlineStr">
         <is>
-          <t>Entrada #90 — pathfinding de uteste até Domain Admins devolveu "Path not found": resultado válido que confirma ausência de caminho neste momento (não uma garantia permanente).</t>
+          <t>Entrada #89 — RootDSE do LDAP exposto por definição de protocolo (não é falha); bind anónimo, listagem SMB e transferência de zona corretamente bloqueados neste domínio.</t>
         </is>
       </c>
       <c r="N17" s="5" t="inlineStr">
         <is>
           <t>⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="O17" s="3" t="inlineStr">
+        <is>
+          <t>Deteção: 🟢 (regra de fábrica 92652, confirmada na #101). Mitigação: parte da informação é exposta por desenho do protocolo; as operações reais com sessão nula foram recusadas (#89).</t>
         </is>
       </c>
     </row>
     <row r="18" ht="110" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Kerberoasting</t>
+          <t>BloodHound — mapeamento de caminhos de ataque em AD</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Ataque a credenciais (Active Directory / Kerberos)</t>
+          <t>Ataque à rede (reconhecimento autenticado / escalação de privilégios, Active Directory)</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Pedido de um Ticket de Serviço (TGS) para uma conta com SPN, usando qualquer conta de domínio autenticada; o ticket vem cifrado com a password da conta de serviço, quebrável offline.</t>
+          <t>Recolha e visualização gráfica das relações de permissões do Active Directory para identificar caminhos possíveis de escalação de privilégio até Domain Admin, a partir de uma conta de baixo privilégio.</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Obter a password de uma conta de serviço (frequentemente privilegiada) através de quebra offline do hash.</t>
+          <t>Encontrar um caminho de escalação de privilégio vertical dentro do domínio.</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>Alta a Crítica (depende do privilégio real da conta de serviço)</t>
+          <t>Crítica se existir caminho; informativa se não existir</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>Confidencialidade, Integridade</t>
+          <t>Confidencialidade, Integridade, Disponibilidade (compromisso total do domínio se o caminho existir e for explorado)</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>Evento 4769 (pedido de TGS) com tipo de cifra RC4 (etype 23) para uma conta de serviço — o único momento observável de todo o ataque.</t>
+          <t>Volume anómalo de consultas LDAP/SMB de uma única conta num curto espaço de tempo — assinatura típica de um collector (SharpHound/bloodhound-python).</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>Passwords longas/aleatórias para contas de serviço; contas de serviço geridas (gMSA); remover SPNs desnecessários; forçar AES em vez de RC4.</t>
+          <t>Princípio do menor privilégio consistente; rever e reverter permissões temporárias; auditorias BloodHound próprias e periódicas (uso defensivo da mesma ferramenta).</t>
         </is>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>Regra dedicada para o Evento 4769 com cifra RC4 — não coberto pelo ruleset genérico de fábrica (confirmado neste lab, Entradas #93-95).</t>
+          <t>Monitorização de volume de consultas LDAP de uma única conta; Microsoft Defender for Identity ou equivalente.</t>
         </is>
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>Rodar imediatamente a password da conta de serviço; rever o que essa conta consegue aceder.</t>
+          <t>Se um caminho for encontrado, corrigir a cadeia de permissões que o permite, não só o nó final.</t>
         </is>
       </c>
       <c r="K18" s="3" t="inlineStr">
         <is>
-          <t>gMSA, SIEM/regra dedicada (Evento 4769 + RC4), Advanced Audit Policy, cofre de segredos.</t>
+          <t>Auditoria periódica com BloodHound (defensiva), Defender for Identity, revisão de grupos privilegiados.</t>
         </is>
       </c>
       <c r="L18" s="3" t="inlineStr">
         <is>
-          <t>ISO 27001 A.5.17, A.8.5 (autenticação segura); NIS2 Art.21; MITRE ATT&amp;CK T1558.003.</t>
+          <t>ISO 27001 A.5.15 (controlo de acesso), A.8.2 (direitos de acesso privilegiado); NIS2 Art.21; MITRE ATT&amp;CK T1087/T1069/T1482.</t>
         </is>
       </c>
       <c r="M18" s="3" t="inlineStr">
         <is>
-          <t>Entrada #91 — conta svc_sql com password Password123, hash TGS quebrado em menos de 1 segundo com hashcat; zero tentativas de login falhadas geradas (invisível ao bloqueio de conta).</t>
+          <t>Entrada #90 — pathfinding de uteste até Domain Admins devolveu "Path not found": resultado válido que confirma ausência de caminho neste momento (não uma garantia permanente).</t>
         </is>
       </c>
       <c r="N18" s="5" t="inlineStr">
         <is>
           <t>⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="O18" s="3" t="inlineStr">
+        <is>
+          <t>Deteção: 🟢 desde a #120 (regra 100021), só para enumeração rápida; a lenta não é coberta (risco #7, Médio provisório). Mitigação: a análise não encontrou caminho da conta de teste até Domain Admins (#90).</t>
         </is>
       </c>
     </row>
     <row r="19" ht="110" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>AS-REP Roasting</t>
+          <t>Kerberoasting</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1826,17 +1852,17 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Pedido da resposta inicial de autenticação Kerberos (AS-REP) para uma conta com pré-autenticação desativada, sem qualquer credencial — o hash devolvido é quebrável offline.</t>
+          <t>Pedido de um Ticket de Serviço (TGS) para uma conta com SPN, usando qualquer conta de domínio autenticada; o ticket vem cifrado com a password da conta de serviço, quebrável offline.</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Obter a password de uma conta vulnerável sem qualquer acesso prévio ao domínio.</t>
-        </is>
-      </c>
-      <c r="E19" s="6" t="inlineStr">
-        <is>
-          <t>Alta (em teoria a mais perigosa das duas variantes Kerberos, por não exigir nenhuma credencial)</t>
+          <t>Obter a password de uma conta de serviço (frequentemente privilegiada) através de quebra offline do hash.</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Alta a Crítica (depende do privilégio real da conta de serviço)</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
@@ -1846,119 +1872,206 @@
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>Evento 4768 (pedido de TGT) sem pré-autenticação correspondente, para contas com DoesNotRequirePreAuth ativo.</t>
+          <t>Evento 4769 (pedido de TGS) com tipo de cifra RC4 (etype 23) para uma conta de serviço — o único momento observável de todo o ataque.</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>Auditar periodicamente Get-ADUser -Filter * -Properties DoesNotRequirePreAuth — raramente deveria estar ativo; password longa/aleatória onde for mesmo necessário.</t>
+          <t>Passwords longas/aleatórias para contas de serviço; contas de serviço geridas (gMSA); remover SPNs desnecessários; forçar AES em vez de RC4.</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>Regra dedicada para o Evento 4768 — não coberto pelo ruleset genérico de fábrica (confirmado neste lab, Entrada #94).</t>
+          <t>Regra dedicada para o Evento 4769 com cifra RC4 — não coberto pelo ruleset genérico de fábrica (confirmado neste lab, Entradas #93-95).</t>
         </is>
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
-          <t>Desativar a definição vulnerável ou rodar a password imediatamente.</t>
+          <t>Rodar imediatamente a password da conta de serviço; rever o que essa conta consegue aceder.</t>
         </is>
       </c>
       <c r="K19" s="3" t="inlineStr">
         <is>
-          <t>Auditoria periódica de AD, SIEM/regra dedicada (Evento 4768), Advanced Audit Policy.</t>
+          <t>gMSA, SIEM/regra dedicada (Evento 4769 + RC4), Advanced Audit Policy, cofre de segredos.</t>
         </is>
       </c>
       <c r="L19" s="3" t="inlineStr">
         <is>
-          <t>ISO 27001 A.5.17, A.8.5; NIS2 Art.21; MITRE ATT&amp;CK T1558.004.</t>
+          <t>ISO 27001 A.5.17, A.8.5 (autenticação segura); NIS2 Art.21; MITRE ATT&amp;CK T1558.003.</t>
         </is>
       </c>
       <c r="M19" s="3" t="inlineStr">
         <is>
-          <t>Entrada #92 — conta svc_legacy com pré-autenticação desativada, hash obtido sem qualquer credencial de domínio; password Welcome123 quebrada em cerca de 2 segundos.</t>
+          <t>Entrada #91 — conta svc_sql com password Password123, hash TGS quebrado em menos de 1 segundo com hashcat; zero tentativas de login falhadas geradas (invisível ao bloqueio de conta).</t>
         </is>
       </c>
       <c r="N19" s="5" t="inlineStr">
         <is>
           <t>⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="O19" s="3" t="inlineStr">
+        <is>
+          <t>Deteção: 🟢 (regra 100011, #95; não reverificada na Fase 9). Mitigação: demonstrada noutras contas (gMSA, #119/#123); não aplicada à svc_sql, mantida fraca como exceção didática (risco #2).</t>
         </is>
       </c>
     </row>
     <row r="20" ht="110" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
+          <t>AS-REP Roasting</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Ataque a credenciais (Active Directory / Kerberos)</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Pedido da resposta inicial de autenticação Kerberos (AS-REP) para uma conta com pré-autenticação desativada, sem qualquer credencial — o hash devolvido é quebrável offline.</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Obter a password de uma conta vulnerável sem qualquer acesso prévio ao domínio.</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>Alta (em teoria a mais perigosa das duas variantes Kerberos, por não exigir nenhuma credencial)</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>Confidencialidade, Integridade</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>Evento 4768 (pedido de TGT) sem pré-autenticação correspondente, para contas com DoesNotRequirePreAuth ativo.</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>Auditar periodicamente Get-ADUser -Filter * -Properties DoesNotRequirePreAuth — raramente deveria estar ativo; password longa/aleatória onde for mesmo necessário.</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>Regra dedicada para o Evento 4768 — não coberto pelo ruleset genérico de fábrica (confirmado neste lab, Entrada #94).</t>
+        </is>
+      </c>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>Desativar a definição vulnerável ou rodar a password imediatamente.</t>
+        </is>
+      </c>
+      <c r="K20" s="3" t="inlineStr">
+        <is>
+          <t>Auditoria periódica de AD, SIEM/regra dedicada (Evento 4768), Advanced Audit Policy.</t>
+        </is>
+      </c>
+      <c r="L20" s="3" t="inlineStr">
+        <is>
+          <t>ISO 27001 A.5.17, A.8.5; NIS2 Art.21; MITRE ATT&amp;CK T1558.004.</t>
+        </is>
+      </c>
+      <c r="M20" s="3" t="inlineStr">
+        <is>
+          <t>Entrada #92 — conta svc_legacy com pré-autenticação desativada, hash obtido sem qualquer credencial de domínio; password Welcome123 quebrada em cerca de 2 segundos.</t>
+        </is>
+      </c>
+      <c r="N20" s="5" t="inlineStr">
+        <is>
+          <t>⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="O20" s="3" t="inlineStr">
+        <is>
+          <t>Deteção: 🟢 (#93/#94; não reverificada na Fase 9). Mitigação: não aplicada à svc_legacy, mantida sem pré-autenticação como exceção didática (risco #2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
           <t>LLMNR / NBT-NS Poisoning (Responder)</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>Ataque à rede (interceção e falsificação de resolução de nomes)</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr">
         <is>
           <t>Resposta falsa a pedidos de resolução de nome multicast (LLMNR/NBT-NS), gerados automaticamente pelo Windows quando a resolução DNS normal falha, capturando a autenticação NTLM que o cliente envia automaticamente ao servidor falso.</t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr">
+      <c r="D21" s="3" t="inlineStr">
         <is>
           <t>Captura de hash de credenciais (NTLMv2), sem exigir nenhum acesso prévio; base para quebra offline ou NTLM relay.</t>
         </is>
       </c>
-      <c r="E20" s="6" t="inlineStr">
+      <c r="E21" s="6" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="F20" s="3" t="inlineStr">
+      <c r="F21" s="3" t="inlineStr">
         <is>
           <t>Confidencialidade (credenciais); Integridade se o hash for reencaminhado (relay) para acesso direto</t>
         </is>
       </c>
-      <c r="G20" s="3" t="inlineStr">
+      <c r="G21" s="3" t="inlineStr">
         <is>
           <t>Tráfego multicast UDP 5355/137 anómalo; respostas a pedidos LLMNR/NBT-NS de origem inesperada; autenticações SMB/NTLM automáticas para nomes que não existem na rede.</t>
         </is>
       </c>
-      <c r="H20" s="3" t="inlineStr">
+      <c r="H21" s="3" t="inlineStr">
         <is>
           <t>Desativar LLMNR e NBT-NS via política de grupo (GPO); usar apenas DNS interno fiável; SMB signing obrigatório para impedir relay.</t>
         </is>
       </c>
-      <c r="I20" s="3" t="inlineStr">
+      <c r="I21" s="3" t="inlineStr">
         <is>
           <t>Monitorização de tráfego LLMNR/NBT-NS na rede; IDS com assinaturas para respostas de ferramentas tipo Responder.</t>
         </is>
       </c>
-      <c r="J20" s="3" t="inlineStr">
+      <c r="J21" s="3" t="inlineStr">
         <is>
           <t>Rodar imediatamente a password da conta cujo hash foi capturado; investigar se houve relay bem-sucedido.</t>
         </is>
       </c>
-      <c r="K20" s="3" t="inlineStr">
+      <c r="K21" s="3" t="inlineStr">
         <is>
           <t>GPO para desativar LLMNR/NBT-NS, SMB signing obrigatório, segmentação de rede, IDS.</t>
         </is>
       </c>
-      <c r="L20" s="3" t="inlineStr">
+      <c r="L21" s="3" t="inlineStr">
         <is>
           <t>ISO 27001 A.8.20 (segurança de redes), A.5.17; NIS2 Art.21; MITRE ATT&amp;CK T1557.001.</t>
         </is>
       </c>
-      <c r="M20" s="3" t="inlineStr">
+      <c r="M21" s="3" t="inlineStr">
         <is>
           <t>Entrada #97 — hash NTLMv2 completo capturado a partir de um simples erro de digitação (\\ficheros) no Windows 11, sem qualquer ação da vítima além do erro de digitação.</t>
         </is>
       </c>
-      <c r="N20" s="5" t="inlineStr">
+      <c r="N21" s="5" t="inlineStr">
         <is>
           <t>⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="O21" s="3" t="inlineStr">
+        <is>
+          <t>Deteção: 🔴. Mitigação: LLMNR/NBT-NS/mDNS desligados (#98), reconfirmado na #106 (risco #3, Baixo).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N20"/>
+  <autoFilter ref="A2:O21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Tabela de ataques: linhas 11, 17 e 18 — controlo efetivamente retestado vs. só verificado antes; 'não reverificada na Fase 9' em destaque
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Lk2S9R4Pvx1JAK73UPgK7J
</commit_message>
<xml_diff>
--- a/tabela-resumo-ataques.xlsx
+++ b/tabela-resumo-ataques.xlsx
@@ -1450,7 +1450,7 @@
       </c>
       <c r="O13" s="3" t="inlineStr">
         <is>
-          <t>Deteção: 🟢 desde a #102. Mitigação: causa corrigida na #104 (FTP só de leitura, PHP desligado na pasta de upload); recusa reconfirmada ao vivo a 2026-10-19 (#129). Por tratar na Fase 10: pasta de upload a 777 e caminhos de escrita anónima (risco #1).</t>
+          <t>Deteção: 🟢 desde a #102. Mitigação: causa corrigida na #104, em duas camadas — (1) FTP anónimo só de leitura: controlo RETESTADO ao vivo a 2026-10-19 (#129: envio recusado com 550 e nada no disco); (2) PHP desligado na pasta de upload: verificado na auditoria da #115, NÃO retestado na Fase 9. Por tratar na Fase 10: pasta de upload a 777 e caminhos de escrita anónima (risco #1).</t>
         </is>
       </c>
     </row>
@@ -1912,7 +1912,7 @@
       </c>
       <c r="O19" s="3" t="inlineStr">
         <is>
-          <t>Deteção: 🟢 (regra 100011, #95; não reverificada na Fase 9). Mitigação: demonstrada noutras contas (gMSA, #119/#123); não aplicada à svc_sql, mantida fraca como exceção didática (risco #2).</t>
+          <t>Deteção: 🟢 — evidência histórica (regra 100011, Fases 6–7, #95); NÃO REVERIFICADA NA FASE 9 (reverificação na Fase 10). Mitigação: demonstrada noutras contas (gMSA, #119/#123); não aplicada à svc_sql, mantida fraca como exceção didática (risco #2).</t>
         </is>
       </c>
     </row>
@@ -1989,7 +1989,7 @@
       </c>
       <c r="O20" s="3" t="inlineStr">
         <is>
-          <t>Deteção: 🟢 (#93/#94; não reverificada na Fase 9). Mitigação: não aplicada à svc_legacy, mantida sem pré-autenticação como exceção didática (risco #2).</t>
+          <t>Deteção: 🟢 — evidência histórica (Fases 6–7; regra validada a 2026-09-22 — ver mapa MITRE, linha 18); NÃO REVERIFICADA NA FASE 9 (reverificação na Fase 10). Mitigação: não aplicada à svc_legacy, mantida sem pré-autenticação como exceção didática (risco #2).</t>
         </is>
       </c>
     </row>

</xml_diff>